<commit_message>
Fixed DTR Export and Template.
</commit_message>
<xml_diff>
--- a/frontend/template/Blank_DTR_Template.xlsx
+++ b/frontend/template/Blank_DTR_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\WIP\Projects\javascript\JS-Portable-DTR-LAN\frontend\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D57FF69-5E36-4E5F-8F5F-A6622A2B5BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A4D465-DA3D-4656-87CA-863B4CCF212B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{643A9BC9-CE66-46F2-AED3-9EEA48CB092B}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$U$64</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$U$63</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="20">
   <si>
     <t>DAILY TIME RECORD</t>
   </si>
@@ -80,6 +80,10 @@
   </si>
   <si>
     <t>VERIFIED as to the prescribed office hours:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I certify on my honor that the above is a true and correct report of the hours of work performed, record of which was made daily at the time of arrival and departure from office.
+</t>
   </si>
 </sst>
 </file>
@@ -500,7 +504,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -664,65 +668,68 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -739,146 +746,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>116206</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>379095</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>10298</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1026" name="Text Box 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCDCE43E-B3A5-EEF8-E0A4-11CA35D14156}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="3601737" y="6510828"/>
-          <a:ext cx="2981480" cy="547970"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:noFill/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="22860" rIns="0" bIns="0" anchor="t" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" i="1">
-              <a:effectLst/>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>I certify on my honor that the above is a true and correct report of the hours of work performed, record of which was made daily at the time of arrival and departure from office.</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-PH" sz="800">
-            <a:effectLst/>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>93345</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>127635</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>19065</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>15446</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Text Box 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E7BA94A1-6D2A-9FE7-D483-FE760A92CA4D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="252953" y="6522257"/>
-          <a:ext cx="3014909" cy="541689"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:noFill/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="22860" rIns="0" bIns="0" anchor="t" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" i="1">
-              <a:effectLst/>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>I certify on my honor that the above is a true and correct report of the hours of work performed, record of which was made daily at the time of arrival and departure from office.</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-PH" sz="800">
-            <a:effectLst/>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1226,18 +1093,18 @@
     </row>
     <row r="3" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B3" s="20"/>
-      <c r="C3" s="79" t="s">
+      <c r="C3" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
       <c r="J3" s="15"/>
       <c r="L3" s="12"/>
-      <c r="M3" s="79" t="s">
+      <c r="M3" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="N3" s="79"/>
-      <c r="O3" s="79"/>
+      <c r="N3" s="78"/>
+      <c r="O3" s="78"/>
       <c r="T3" s="27"/>
     </row>
     <row r="4" spans="2:20" x14ac:dyDescent="0.2">
@@ -1297,49 +1164,49 @@
     <row r="8" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20"/>
       <c r="C8" s="50"/>
-      <c r="D8" s="66"/>
-      <c r="E8" s="66"/>
-      <c r="F8" s="66"/>
-      <c r="G8" s="66"/>
-      <c r="H8" s="66"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
       <c r="I8" s="50"/>
       <c r="J8" s="29"/>
       <c r="K8" s="30"/>
       <c r="L8" s="31"/>
       <c r="M8" s="50"/>
-      <c r="N8" s="66">
+      <c r="N8" s="72">
         <f>D8</f>
         <v>0</v>
       </c>
-      <c r="O8" s="66"/>
-      <c r="P8" s="66"/>
-      <c r="Q8" s="66"/>
-      <c r="R8" s="66"/>
+      <c r="O8" s="72"/>
+      <c r="P8" s="72"/>
+      <c r="Q8" s="72"/>
+      <c r="R8" s="72"/>
       <c r="S8" s="50"/>
       <c r="T8" s="27"/>
     </row>
     <row r="9" spans="2:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="20"/>
-      <c r="C9" s="73" t="s">
+      <c r="C9" s="81" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
-      <c r="F9" s="74"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="74"/>
-      <c r="I9" s="73"/>
+      <c r="D9" s="82"/>
+      <c r="E9" s="82"/>
+      <c r="F9" s="82"/>
+      <c r="G9" s="82"/>
+      <c r="H9" s="82"/>
+      <c r="I9" s="81"/>
       <c r="J9" s="15"/>
       <c r="L9" s="12"/>
-      <c r="M9" s="73" t="s">
+      <c r="M9" s="81" t="s">
         <v>9</v>
       </c>
-      <c r="N9" s="74"/>
-      <c r="O9" s="74"/>
-      <c r="P9" s="74"/>
-      <c r="Q9" s="74"/>
-      <c r="R9" s="74"/>
-      <c r="S9" s="73"/>
+      <c r="N9" s="82"/>
+      <c r="O9" s="82"/>
+      <c r="P9" s="82"/>
+      <c r="Q9" s="82"/>
+      <c r="R9" s="82"/>
+      <c r="S9" s="81"/>
       <c r="T9" s="27"/>
     </row>
     <row r="10" spans="2:20" ht="13.2" x14ac:dyDescent="0.25">
@@ -1365,38 +1232,38 @@
     </row>
     <row r="11" spans="2:20" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="20"/>
-      <c r="C11" s="71" t="s">
+      <c r="C11" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="71"/>
-      <c r="E11" s="71"/>
-      <c r="F11" s="80"/>
-      <c r="G11" s="80"/>
-      <c r="H11" s="80"/>
-      <c r="I11" s="80"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="73"/>
+      <c r="G11" s="73"/>
+      <c r="H11" s="73"/>
+      <c r="I11" s="73"/>
       <c r="J11" s="15"/>
       <c r="L11" s="12"/>
-      <c r="M11" s="71" t="s">
+      <c r="M11" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="N11" s="71"/>
-      <c r="O11" s="71"/>
-      <c r="P11" s="80">
+      <c r="N11" s="74"/>
+      <c r="O11" s="74"/>
+      <c r="P11" s="73">
         <f>F11</f>
         <v>0</v>
       </c>
-      <c r="Q11" s="80"/>
-      <c r="R11" s="80"/>
-      <c r="S11" s="80"/>
+      <c r="Q11" s="73"/>
+      <c r="R11" s="73"/>
+      <c r="S11" s="73"/>
       <c r="T11" s="27"/>
     </row>
     <row r="12" spans="2:20" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B12" s="20"/>
-      <c r="C12" s="72" t="s">
+      <c r="C12" s="79" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="72"/>
-      <c r="E12" s="72"/>
+      <c r="D12" s="79"/>
+      <c r="E12" s="79"/>
       <c r="G12" s="36" t="s">
         <v>15</v>
       </c>
@@ -1404,11 +1271,11 @@
       <c r="I12" s="38"/>
       <c r="J12" s="15"/>
       <c r="L12" s="12"/>
-      <c r="M12" s="72" t="s">
+      <c r="M12" s="79" t="s">
         <v>12</v>
       </c>
-      <c r="N12" s="72"/>
-      <c r="O12" s="72"/>
+      <c r="N12" s="79"/>
+      <c r="O12" s="79"/>
       <c r="Q12" s="36" t="s">
         <v>15</v>
       </c>
@@ -1418,11 +1285,11 @@
     </row>
     <row r="13" spans="2:20" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B13" s="20"/>
-      <c r="C13" s="72" t="s">
+      <c r="C13" s="79" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="72"/>
-      <c r="E13" s="72"/>
+      <c r="D13" s="79"/>
+      <c r="E13" s="79"/>
       <c r="G13" s="36" t="s">
         <v>1</v>
       </c>
@@ -1430,11 +1297,11 @@
       <c r="I13" s="38"/>
       <c r="J13" s="15"/>
       <c r="L13" s="12"/>
-      <c r="M13" s="72" t="s">
+      <c r="M13" s="79" t="s">
         <v>13</v>
       </c>
-      <c r="N13" s="72"/>
-      <c r="O13" s="72"/>
+      <c r="N13" s="79"/>
+      <c r="O13" s="79"/>
       <c r="Q13" s="36" t="s">
         <v>1</v>
       </c>
@@ -1464,43 +1331,43 @@
     </row>
     <row r="15" spans="2:20" ht="13.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B15" s="20"/>
-      <c r="C15" s="81" t="s">
+      <c r="C15" s="70" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="63" t="s">
+      <c r="D15" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="64"/>
-      <c r="F15" s="63" t="s">
+      <c r="E15" s="68"/>
+      <c r="F15" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="G15" s="64"/>
-      <c r="H15" s="63" t="s">
+      <c r="G15" s="68"/>
+      <c r="H15" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="I15" s="70"/>
+      <c r="I15" s="67"/>
       <c r="J15" s="6"/>
       <c r="L15" s="6"/>
-      <c r="M15" s="81" t="s">
+      <c r="M15" s="70" t="s">
         <v>14</v>
       </c>
-      <c r="N15" s="63" t="s">
+      <c r="N15" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="O15" s="64"/>
-      <c r="P15" s="63" t="s">
+      <c r="O15" s="68"/>
+      <c r="P15" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="Q15" s="64"/>
-      <c r="R15" s="63" t="s">
+      <c r="Q15" s="68"/>
+      <c r="R15" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="S15" s="65"/>
+      <c r="S15" s="71"/>
       <c r="T15" s="27"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B16" s="20"/>
-      <c r="C16" s="64"/>
+      <c r="C16" s="68"/>
       <c r="D16" s="44" t="s">
         <v>5</v>
       </c>
@@ -1521,7 +1388,7 @@
       </c>
       <c r="J16" s="6"/>
       <c r="L16" s="6"/>
-      <c r="M16" s="64"/>
+      <c r="M16" s="68"/>
       <c r="N16" s="44" t="s">
         <v>5</v>
       </c>
@@ -3074,28 +2941,88 @@
       <c r="L49" s="12"/>
       <c r="T49" s="27"/>
     </row>
-    <row r="50" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:20" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="20"/>
+      <c r="C50" s="83" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" s="83"/>
+      <c r="E50" s="83"/>
+      <c r="F50" s="83"/>
+      <c r="G50" s="83"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="83"/>
       <c r="J50" s="15"/>
       <c r="L50" s="12"/>
+      <c r="M50" s="83" t="s">
+        <v>19</v>
+      </c>
+      <c r="N50" s="83"/>
+      <c r="O50" s="83"/>
+      <c r="P50" s="83"/>
+      <c r="Q50" s="83"/>
+      <c r="R50" s="83"/>
+      <c r="S50" s="83"/>
       <c r="T50" s="27"/>
     </row>
     <row r="51" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B51" s="20"/>
+      <c r="C51" s="83"/>
+      <c r="D51" s="83"/>
+      <c r="E51" s="83"/>
+      <c r="F51" s="83"/>
+      <c r="G51" s="83"/>
+      <c r="H51" s="83"/>
+      <c r="I51" s="83"/>
       <c r="J51" s="15"/>
       <c r="L51" s="12"/>
+      <c r="M51" s="83"/>
+      <c r="N51" s="83"/>
+      <c r="O51" s="83"/>
+      <c r="P51" s="83"/>
+      <c r="Q51" s="83"/>
+      <c r="R51" s="83"/>
+      <c r="S51" s="83"/>
       <c r="T51" s="27"/>
     </row>
     <row r="52" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B52" s="20"/>
+      <c r="C52" s="83"/>
+      <c r="D52" s="83"/>
+      <c r="E52" s="83"/>
+      <c r="F52" s="83"/>
+      <c r="G52" s="83"/>
+      <c r="H52" s="83"/>
+      <c r="I52" s="83"/>
       <c r="J52" s="15"/>
       <c r="L52" s="12"/>
+      <c r="M52" s="83"/>
+      <c r="N52" s="83"/>
+      <c r="O52" s="83"/>
+      <c r="P52" s="83"/>
+      <c r="Q52" s="83"/>
+      <c r="R52" s="83"/>
+      <c r="S52" s="83"/>
       <c r="T52" s="27"/>
     </row>
     <row r="53" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B53" s="20"/>
+      <c r="C53" s="83"/>
+      <c r="D53" s="83"/>
+      <c r="E53" s="83"/>
+      <c r="F53" s="83"/>
+      <c r="G53" s="83"/>
+      <c r="H53" s="83"/>
+      <c r="I53" s="83"/>
       <c r="J53" s="15"/>
       <c r="L53" s="12"/>
+      <c r="M53" s="83"/>
+      <c r="N53" s="83"/>
+      <c r="O53" s="83"/>
+      <c r="P53" s="83"/>
+      <c r="Q53" s="83"/>
+      <c r="R53" s="83"/>
+      <c r="S53" s="83"/>
       <c r="T53" s="27"/>
     </row>
     <row r="54" spans="2:20" x14ac:dyDescent="0.2">
@@ -3106,21 +3033,21 @@
     </row>
     <row r="55" spans="2:20" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B55" s="20"/>
-      <c r="D55" s="82"/>
-      <c r="E55" s="82"/>
-      <c r="F55" s="82"/>
-      <c r="G55" s="82"/>
-      <c r="H55" s="82"/>
+      <c r="D55" s="80"/>
+      <c r="E55" s="80"/>
+      <c r="F55" s="80"/>
+      <c r="G55" s="80"/>
+      <c r="H55" s="80"/>
       <c r="J55" s="15"/>
       <c r="L55" s="12"/>
-      <c r="N55" s="82">
+      <c r="N55" s="80">
         <f>D55</f>
         <v>0</v>
       </c>
-      <c r="O55" s="82"/>
-      <c r="P55" s="82"/>
-      <c r="Q55" s="82"/>
-      <c r="R55" s="82"/>
+      <c r="O55" s="80"/>
+      <c r="P55" s="80"/>
+      <c r="Q55" s="80"/>
+      <c r="R55" s="80"/>
       <c r="T55" s="27"/>
     </row>
     <row r="56" spans="2:20" x14ac:dyDescent="0.2">
@@ -3157,26 +3084,26 @@
     </row>
     <row r="58" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B58" s="20"/>
-      <c r="C58" s="78" t="s">
+      <c r="C58" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="D58" s="78"/>
-      <c r="E58" s="78"/>
-      <c r="F58" s="78"/>
-      <c r="G58" s="78"/>
-      <c r="H58" s="78"/>
-      <c r="I58" s="78"/>
+      <c r="D58" s="69"/>
+      <c r="E58" s="69"/>
+      <c r="F58" s="69"/>
+      <c r="G58" s="69"/>
+      <c r="H58" s="69"/>
+      <c r="I58" s="69"/>
       <c r="J58" s="15"/>
       <c r="L58" s="20"/>
-      <c r="M58" s="78" t="s">
+      <c r="M58" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="N58" s="78"/>
-      <c r="O58" s="78"/>
-      <c r="P58" s="78"/>
-      <c r="Q58" s="78"/>
-      <c r="R58" s="78"/>
-      <c r="S58" s="78"/>
+      <c r="N58" s="69"/>
+      <c r="O58" s="69"/>
+      <c r="P58" s="69"/>
+      <c r="Q58" s="69"/>
+      <c r="R58" s="69"/>
+      <c r="S58" s="69"/>
       <c r="T58" s="15"/>
     </row>
     <row r="59" spans="2:20" x14ac:dyDescent="0.2">
@@ -3193,43 +3120,43 @@
     </row>
     <row r="61" spans="2:20" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B61" s="20"/>
-      <c r="D61" s="66"/>
-      <c r="E61" s="66"/>
-      <c r="F61" s="66"/>
-      <c r="G61" s="66"/>
-      <c r="H61" s="66"/>
+      <c r="D61" s="72"/>
+      <c r="E61" s="72"/>
+      <c r="F61" s="72"/>
+      <c r="G61" s="72"/>
+      <c r="H61" s="72"/>
       <c r="J61" s="15"/>
       <c r="L61" s="20"/>
-      <c r="N61" s="66">
+      <c r="N61" s="72">
         <f>D61</f>
         <v>0</v>
       </c>
-      <c r="O61" s="66"/>
-      <c r="P61" s="66"/>
-      <c r="Q61" s="66"/>
-      <c r="R61" s="66"/>
+      <c r="O61" s="72"/>
+      <c r="P61" s="72"/>
+      <c r="Q61" s="72"/>
+      <c r="R61" s="72"/>
       <c r="T61" s="15"/>
     </row>
     <row r="62" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B62" s="20"/>
-      <c r="D62" s="67" t="s">
+      <c r="D62" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="E62" s="68"/>
-      <c r="F62" s="68"/>
-      <c r="G62" s="68"/>
-      <c r="H62" s="68"/>
+      <c r="E62" s="64"/>
+      <c r="F62" s="64"/>
+      <c r="G62" s="64"/>
+      <c r="H62" s="64"/>
       <c r="I62" s="8"/>
       <c r="J62" s="22"/>
       <c r="K62" s="8"/>
       <c r="L62" s="20"/>
-      <c r="N62" s="67" t="s">
+      <c r="N62" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="O62" s="68"/>
-      <c r="P62" s="68"/>
-      <c r="Q62" s="68"/>
-      <c r="R62" s="68"/>
+      <c r="O62" s="64"/>
+      <c r="P62" s="64"/>
+      <c r="Q62" s="64"/>
+      <c r="R62" s="64"/>
       <c r="S62" s="8"/>
       <c r="T62" s="22"/>
     </row>
@@ -3255,17 +3182,17 @@
       <c r="T63" s="49"/>
     </row>
     <row r="64" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="H64" s="69"/>
-      <c r="I64" s="69"/>
+      <c r="H64" s="65"/>
+      <c r="I64" s="65"/>
       <c r="J64" s="24"/>
       <c r="K64" s="24"/>
       <c r="L64" s="2"/>
-      <c r="R64" s="69"/>
-      <c r="S64" s="69"/>
+      <c r="R64" s="65"/>
+      <c r="S64" s="65"/>
       <c r="T64" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="38">
     <mergeCell ref="M13:O13"/>
     <mergeCell ref="D55:H55"/>
     <mergeCell ref="N55:R55"/>
@@ -3275,6 +3202,9 @@
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="M9:S9"/>
+    <mergeCell ref="M12:O12"/>
+    <mergeCell ref="M50:S53"/>
+    <mergeCell ref="C50:I53"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="M2:O2"/>
     <mergeCell ref="D5:H5"/>
@@ -3286,7 +3216,6 @@
     <mergeCell ref="F11:I11"/>
     <mergeCell ref="P11:S11"/>
     <mergeCell ref="M11:O11"/>
-    <mergeCell ref="M12:O12"/>
     <mergeCell ref="D62:H62"/>
     <mergeCell ref="N62:R62"/>
     <mergeCell ref="H64:I64"/>
@@ -3307,6 +3236,5 @@
   <pageMargins left="0.54" right="0.45" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup scale="96" orientation="portrait" horizontalDpi="120" verticalDpi="144" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implementing Attendance Corrections feature.
</commit_message>
<xml_diff>
--- a/frontend/template/Blank_DTR_Template.xlsx
+++ b/frontend/template/Blank_DTR_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\WIP\Projects\javascript\JS-Portable-DTR-LAN\frontend\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A4D465-DA3D-4656-87CA-863B4CCF212B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD18365-24AC-4966-87E4-84DA84B9D9C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{643A9BC9-CE66-46F2-AED3-9EEA48CB092B}"/>
   </bookViews>
@@ -597,9 +597,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -730,6 +727,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1073,18 +1073,18 @@
   <sheetData>
     <row r="2" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B2" s="17"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
       <c r="F2" s="18"/>
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
       <c r="I2" s="18"/>
       <c r="J2" s="19"/>
       <c r="L2" s="25"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="76"/>
-      <c r="O2" s="76"/>
+      <c r="M2" s="75"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="75"/>
       <c r="P2" s="18"/>
       <c r="Q2" s="18"/>
       <c r="R2" s="18"/>
@@ -1093,18 +1093,18 @@
     </row>
     <row r="3" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B3" s="20"/>
-      <c r="C3" s="78" t="s">
+      <c r="C3" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="78"/>
-      <c r="E3" s="78"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
       <c r="J3" s="15"/>
       <c r="L3" s="12"/>
-      <c r="M3" s="78" t="s">
+      <c r="M3" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="N3" s="78"/>
-      <c r="O3" s="78"/>
+      <c r="N3" s="77"/>
+      <c r="O3" s="77"/>
       <c r="T3" s="27"/>
     </row>
     <row r="4" spans="2:20" x14ac:dyDescent="0.2">
@@ -1121,22 +1121,22 @@
     </row>
     <row r="5" spans="2:20" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="B5" s="20"/>
-      <c r="D5" s="77" t="s">
+      <c r="D5" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="77"/>
-      <c r="F5" s="77"/>
-      <c r="G5" s="77"/>
-      <c r="H5" s="77"/>
+      <c r="E5" s="76"/>
+      <c r="F5" s="76"/>
+      <c r="G5" s="76"/>
+      <c r="H5" s="76"/>
       <c r="J5" s="15"/>
       <c r="L5" s="12"/>
-      <c r="N5" s="77" t="s">
+      <c r="N5" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="O5" s="77"/>
-      <c r="P5" s="77"/>
-      <c r="Q5" s="77"/>
-      <c r="R5" s="77"/>
+      <c r="O5" s="76"/>
+      <c r="P5" s="76"/>
+      <c r="Q5" s="76"/>
+      <c r="R5" s="76"/>
       <c r="T5" s="27"/>
     </row>
     <row r="6" spans="2:20" ht="9.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1163,50 +1163,50 @@
     </row>
     <row r="8" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="72"/>
-      <c r="E8" s="72"/>
-      <c r="F8" s="72"/>
-      <c r="G8" s="72"/>
-      <c r="H8" s="72"/>
-      <c r="I8" s="50"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="71"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="71"/>
+      <c r="G8" s="71"/>
+      <c r="H8" s="71"/>
+      <c r="I8" s="49"/>
       <c r="J8" s="29"/>
       <c r="K8" s="30"/>
       <c r="L8" s="31"/>
-      <c r="M8" s="50"/>
-      <c r="N8" s="72">
-        <f>D8</f>
-        <v>0</v>
-      </c>
-      <c r="O8" s="72"/>
-      <c r="P8" s="72"/>
-      <c r="Q8" s="72"/>
-      <c r="R8" s="72"/>
-      <c r="S8" s="50"/>
+      <c r="M8" s="49"/>
+      <c r="N8" s="71" t="str">
+        <f>IF(D8="","",D8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="71"/>
+      <c r="P8" s="71"/>
+      <c r="Q8" s="71"/>
+      <c r="R8" s="71"/>
+      <c r="S8" s="49"/>
       <c r="T8" s="27"/>
     </row>
     <row r="9" spans="2:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="20"/>
-      <c r="C9" s="81" t="s">
+      <c r="C9" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="82"/>
-      <c r="E9" s="82"/>
-      <c r="F9" s="82"/>
-      <c r="G9" s="82"/>
-      <c r="H9" s="82"/>
-      <c r="I9" s="81"/>
+      <c r="D9" s="81"/>
+      <c r="E9" s="81"/>
+      <c r="F9" s="81"/>
+      <c r="G9" s="81"/>
+      <c r="H9" s="81"/>
+      <c r="I9" s="80"/>
       <c r="J9" s="15"/>
       <c r="L9" s="12"/>
-      <c r="M9" s="81" t="s">
+      <c r="M9" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="N9" s="82"/>
-      <c r="O9" s="82"/>
-      <c r="P9" s="82"/>
-      <c r="Q9" s="82"/>
-      <c r="R9" s="82"/>
-      <c r="S9" s="81"/>
+      <c r="N9" s="81"/>
+      <c r="O9" s="81"/>
+      <c r="P9" s="81"/>
+      <c r="Q9" s="81"/>
+      <c r="R9" s="81"/>
+      <c r="S9" s="80"/>
       <c r="T9" s="27"/>
     </row>
     <row r="10" spans="2:20" ht="13.2" x14ac:dyDescent="0.25">
@@ -1232,81 +1232,87 @@
     </row>
     <row r="11" spans="2:20" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="20"/>
-      <c r="C11" s="74" t="s">
+      <c r="C11" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="74"/>
-      <c r="E11" s="74"/>
-      <c r="F11" s="73"/>
-      <c r="G11" s="73"/>
-      <c r="H11" s="73"/>
-      <c r="I11" s="73"/>
+      <c r="D11" s="73"/>
+      <c r="E11" s="73"/>
+      <c r="F11" s="72"/>
+      <c r="G11" s="72"/>
+      <c r="H11" s="72"/>
+      <c r="I11" s="72"/>
       <c r="J11" s="15"/>
       <c r="L11" s="12"/>
-      <c r="M11" s="74" t="s">
+      <c r="M11" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="N11" s="74"/>
-      <c r="O11" s="74"/>
-      <c r="P11" s="73">
-        <f>F11</f>
-        <v>0</v>
-      </c>
-      <c r="Q11" s="73"/>
-      <c r="R11" s="73"/>
-      <c r="S11" s="73"/>
+      <c r="N11" s="73"/>
+      <c r="O11" s="73"/>
+      <c r="P11" s="72" t="str">
+        <f>IF(F11="","",F11)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="72"/>
+      <c r="R11" s="72"/>
+      <c r="S11" s="72"/>
       <c r="T11" s="27"/>
     </row>
     <row r="12" spans="2:20" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B12" s="20"/>
-      <c r="C12" s="79" t="s">
+      <c r="C12" s="78" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="79"/>
-      <c r="E12" s="79"/>
+      <c r="D12" s="78"/>
+      <c r="E12" s="78"/>
       <c r="G12" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="38"/>
-      <c r="I12" s="38"/>
+      <c r="H12" s="83"/>
+      <c r="I12" s="83"/>
       <c r="J12" s="15"/>
       <c r="L12" s="12"/>
-      <c r="M12" s="79" t="s">
+      <c r="M12" s="78" t="s">
         <v>12</v>
       </c>
-      <c r="N12" s="79"/>
-      <c r="O12" s="79"/>
+      <c r="N12" s="78"/>
+      <c r="O12" s="78"/>
       <c r="Q12" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="R12" s="38"/>
-      <c r="S12" s="38"/>
+      <c r="R12" s="83" t="str">
+        <f>IF(H12="","",H12)</f>
+        <v/>
+      </c>
+      <c r="S12" s="83"/>
       <c r="T12" s="27"/>
     </row>
     <row r="13" spans="2:20" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B13" s="20"/>
-      <c r="C13" s="79" t="s">
+      <c r="C13" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="79"/>
-      <c r="E13" s="79"/>
+      <c r="D13" s="78"/>
+      <c r="E13" s="78"/>
       <c r="G13" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="H13" s="38"/>
-      <c r="I13" s="38"/>
+      <c r="H13" s="83"/>
+      <c r="I13" s="83"/>
       <c r="J13" s="15"/>
       <c r="L13" s="12"/>
-      <c r="M13" s="79" t="s">
+      <c r="M13" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="N13" s="79"/>
-      <c r="O13" s="79"/>
+      <c r="N13" s="78"/>
+      <c r="O13" s="78"/>
       <c r="Q13" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="R13" s="38"/>
-      <c r="S13" s="38"/>
+      <c r="R13" s="83" t="str">
+        <f>IF(H13="","",H13)</f>
+        <v/>
+      </c>
+      <c r="S13" s="83"/>
       <c r="T13" s="27"/>
     </row>
     <row r="14" spans="2:20" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
@@ -1331,1570 +1337,1570 @@
     </row>
     <row r="15" spans="2:20" ht="13.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B15" s="20"/>
-      <c r="C15" s="70" t="s">
+      <c r="C15" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="66" t="s">
+      <c r="D15" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="68"/>
-      <c r="F15" s="66" t="s">
+      <c r="E15" s="67"/>
+      <c r="F15" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="G15" s="68"/>
-      <c r="H15" s="66" t="s">
+      <c r="G15" s="67"/>
+      <c r="H15" s="65" t="s">
         <v>16</v>
       </c>
-      <c r="I15" s="67"/>
+      <c r="I15" s="66"/>
       <c r="J15" s="6"/>
       <c r="L15" s="6"/>
-      <c r="M15" s="70" t="s">
+      <c r="M15" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="N15" s="66" t="s">
+      <c r="N15" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="O15" s="68"/>
-      <c r="P15" s="66" t="s">
+      <c r="O15" s="67"/>
+      <c r="P15" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="Q15" s="68"/>
-      <c r="R15" s="66" t="s">
+      <c r="Q15" s="67"/>
+      <c r="R15" s="65" t="s">
         <v>16</v>
       </c>
-      <c r="S15" s="71"/>
+      <c r="S15" s="70"/>
       <c r="T15" s="27"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B16" s="20"/>
-      <c r="C16" s="68"/>
-      <c r="D16" s="44" t="s">
+      <c r="C16" s="67"/>
+      <c r="D16" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="45" t="s">
+      <c r="E16" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F16" s="44" t="s">
+      <c r="F16" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="45" t="s">
+      <c r="G16" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="H16" s="44" t="s">
+      <c r="H16" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="I16" s="41" t="s">
+      <c r="I16" s="40" t="s">
         <v>7</v>
       </c>
       <c r="J16" s="6"/>
       <c r="L16" s="6"/>
-      <c r="M16" s="68"/>
-      <c r="N16" s="44" t="s">
+      <c r="M16" s="67"/>
+      <c r="N16" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="O16" s="45" t="s">
+      <c r="O16" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="P16" s="44" t="s">
+      <c r="P16" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="Q16" s="45" t="s">
+      <c r="Q16" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="R16" s="44" t="s">
+      <c r="R16" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="S16" s="40" t="s">
+      <c r="S16" s="39" t="s">
         <v>7</v>
       </c>
       <c r="T16" s="27"/>
     </row>
     <row r="17" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B17" s="20"/>
-      <c r="C17" s="45">
+      <c r="C17" s="44">
         <v>1</v>
       </c>
-      <c r="D17" s="52"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="52"/>
-      <c r="G17" s="53"/>
-      <c r="H17" s="54" t="str">
-        <f>IFERROR(IF(COUNT(D17:G17)&lt;4, "-", INT(MAX(0, (8/24 - ((E17-D17)+(G17-F17))) * 24))), "-")</f>
-        <v>-</v>
-      </c>
-      <c r="I17" s="56" t="str">
-        <f>IFERROR(IF(COUNT(D17:G17)&lt;4, "-", ROUND(MOD(MAX(0, (8/24 - ((E17-D17)+(G17-F17))) * 24), 1) * 60, 0)), "-")</f>
-        <v>-</v>
+      <c r="D17" s="51"/>
+      <c r="E17" s="52"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="52"/>
+      <c r="H17" s="53" t="str">
+        <f>IFERROR(IF(COUNT(D17:G17)&lt;4, "", INT(MAX(0, (8/24 - ((E17-D17)+(G17-F17))) * 24))), "")</f>
+        <v/>
+      </c>
+      <c r="I17" s="55" t="str">
+        <f>IFERROR(IF(COUNT(D17:G17)&lt;4, "", ROUND(MOD(MAX(0, (8/24 - ((E17-D17)+(G17-F17))) * 24), 1) * 60, 0)), "")</f>
+        <v/>
       </c>
       <c r="J17" s="6"/>
       <c r="L17" s="6"/>
-      <c r="M17" s="45">
+      <c r="M17" s="44">
         <v>1</v>
       </c>
-      <c r="N17" s="52">
-        <f t="shared" ref="N17:S17" si="0">D17</f>
-        <v>0</v>
-      </c>
-      <c r="O17" s="53">
+      <c r="N17" s="51" t="str">
+        <f>IF(OR(D17="",D17=0),"",D17)</f>
+        <v/>
+      </c>
+      <c r="O17" s="52" t="str">
+        <f>IF(OR(E17="",E17=0),"",E17)</f>
+        <v/>
+      </c>
+      <c r="P17" s="51" t="str">
+        <f>IF(OR(F17="",F17=0),"",F17)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="52" t="str">
+        <f>IF(OR(G17="",G17=0),"",G17)</f>
+        <v/>
+      </c>
+      <c r="R17" s="53" t="str">
+        <f t="shared" ref="R17:S17" si="0">H17</f>
+        <v/>
+      </c>
+      <c r="S17" s="54" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="P17" s="52">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Q17" s="53">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R17" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="S17" s="55" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T17" s="27"/>
     </row>
     <row r="18" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B18" s="20"/>
-      <c r="C18" s="45">
+      <c r="C18" s="44">
         <v>2</v>
       </c>
-      <c r="D18" s="52"/>
-      <c r="E18" s="53"/>
-      <c r="F18" s="52"/>
-      <c r="G18" s="53"/>
-      <c r="H18" s="54" t="str">
-        <f t="shared" ref="H18:H47" si="1">IFERROR(IF(COUNT(D18:G18)&lt;4, "-", INT(MAX(0, (8/24 - ((E18-D18)+(G18-F18))) * 24))), "-")</f>
-        <v>-</v>
-      </c>
-      <c r="I18" s="56" t="str">
-        <f t="shared" ref="I18:I47" si="2">IFERROR(IF(COUNT(D18:G18)&lt;4, "-", ROUND(MOD(MAX(0, (8/24 - ((E18-D18)+(G18-F18))) * 24), 1) * 60, 0)), "-")</f>
-        <v>-</v>
+      <c r="D18" s="51"/>
+      <c r="E18" s="52"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="52"/>
+      <c r="H18" s="53" t="str">
+        <f t="shared" ref="H18:H47" si="1">IFERROR(IF(COUNT(D18:G18)&lt;4, "", INT(MAX(0, (8/24 - ((E18-D18)+(G18-F18))) * 24))), "")</f>
+        <v/>
+      </c>
+      <c r="I18" s="55" t="str">
+        <f t="shared" ref="I18:I47" si="2">IFERROR(IF(COUNT(D18:G18)&lt;4, "", ROUND(MOD(MAX(0, (8/24 - ((E18-D18)+(G18-F18))) * 24), 1) * 60, 0)), "")</f>
+        <v/>
       </c>
       <c r="J18" s="6"/>
       <c r="L18" s="6"/>
-      <c r="M18" s="45">
+      <c r="M18" s="44">
         <v>2</v>
       </c>
-      <c r="N18" s="52">
-        <f t="shared" ref="N18:N47" si="3">D18</f>
-        <v>0</v>
-      </c>
-      <c r="O18" s="53">
-        <f t="shared" ref="O18:O47" si="4">E18</f>
-        <v>0</v>
-      </c>
-      <c r="P18" s="52">
-        <f t="shared" ref="P18:P47" si="5">F18</f>
-        <v>0</v>
-      </c>
-      <c r="Q18" s="53">
-        <f t="shared" ref="Q18:Q47" si="6">G18</f>
-        <v>0</v>
-      </c>
-      <c r="R18" s="54" t="str">
+      <c r="N18" s="51" t="str">
+        <f t="shared" ref="N18:N47" si="3">IF(OR(D18="",D18=0),"",D18)</f>
+        <v/>
+      </c>
+      <c r="O18" s="52" t="str">
+        <f t="shared" ref="O18:O47" si="4">IF(OR(E18="",E18=0),"",E18)</f>
+        <v/>
+      </c>
+      <c r="P18" s="51" t="str">
+        <f t="shared" ref="P18:P47" si="5">IF(OR(F18="",F18=0),"",F18)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="52" t="str">
+        <f t="shared" ref="Q18:Q47" si="6">IF(OR(G18="",G18=0),"",G18)</f>
+        <v/>
+      </c>
+      <c r="R18" s="53" t="str">
         <f t="shared" ref="R18:R47" si="7">H18</f>
-        <v>-</v>
-      </c>
-      <c r="S18" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S18" s="54" t="str">
         <f t="shared" ref="S18:S47" si="8">I18</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T18" s="27"/>
     </row>
     <row r="19" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B19" s="20"/>
-      <c r="C19" s="45">
+      <c r="C19" s="44">
         <v>3</v>
       </c>
-      <c r="D19" s="52"/>
-      <c r="E19" s="53"/>
-      <c r="F19" s="52"/>
-      <c r="G19" s="53"/>
-      <c r="H19" s="54" t="str">
+      <c r="D19" s="51"/>
+      <c r="E19" s="52"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I19" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I19" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J19" s="6"/>
       <c r="L19" s="6"/>
-      <c r="M19" s="45">
+      <c r="M19" s="44">
         <v>3</v>
       </c>
-      <c r="N19" s="52">
+      <c r="N19" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O19" s="53">
+        <v/>
+      </c>
+      <c r="O19" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P19" s="52">
+        <v/>
+      </c>
+      <c r="P19" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q19" s="53">
+        <v/>
+      </c>
+      <c r="Q19" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R19" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R19" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S19" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S19" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T19" s="27"/>
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B20" s="20"/>
-      <c r="C20" s="45">
+      <c r="C20" s="44">
         <v>4</v>
       </c>
-      <c r="D20" s="52"/>
-      <c r="E20" s="53"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="53"/>
-      <c r="H20" s="54" t="str">
+      <c r="D20" s="51"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I20" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I20" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J20" s="6"/>
       <c r="L20" s="6"/>
-      <c r="M20" s="45">
+      <c r="M20" s="44">
         <v>4</v>
       </c>
-      <c r="N20" s="52">
+      <c r="N20" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O20" s="53">
+        <v/>
+      </c>
+      <c r="O20" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P20" s="52">
+        <v/>
+      </c>
+      <c r="P20" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q20" s="53">
+        <v/>
+      </c>
+      <c r="Q20" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R20" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R20" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S20" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S20" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T20" s="27"/>
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B21" s="20"/>
-      <c r="C21" s="45">
+      <c r="C21" s="44">
         <v>5</v>
       </c>
-      <c r="D21" s="52"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="52"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="54" t="str">
+      <c r="D21" s="51"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I21" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I21" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J21" s="6"/>
       <c r="L21" s="6"/>
-      <c r="M21" s="45">
+      <c r="M21" s="44">
         <v>5</v>
       </c>
-      <c r="N21" s="52">
+      <c r="N21" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O21" s="53">
+        <v/>
+      </c>
+      <c r="O21" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P21" s="52">
+        <v/>
+      </c>
+      <c r="P21" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q21" s="53">
+        <v/>
+      </c>
+      <c r="Q21" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R21" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R21" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S21" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S21" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T21" s="27"/>
     </row>
     <row r="22" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B22" s="20"/>
-      <c r="C22" s="45">
+      <c r="C22" s="44">
         <v>6</v>
       </c>
-      <c r="D22" s="52"/>
-      <c r="E22" s="53"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="53"/>
-      <c r="H22" s="54" t="str">
+      <c r="D22" s="51"/>
+      <c r="E22" s="52"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
+      <c r="H22" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I22" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I22" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J22" s="6"/>
       <c r="L22" s="6"/>
-      <c r="M22" s="45">
+      <c r="M22" s="44">
         <v>6</v>
       </c>
-      <c r="N22" s="52">
+      <c r="N22" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O22" s="53">
+        <v/>
+      </c>
+      <c r="O22" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P22" s="52">
+        <v/>
+      </c>
+      <c r="P22" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q22" s="53">
+        <v/>
+      </c>
+      <c r="Q22" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R22" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R22" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S22" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S22" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T22" s="27"/>
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B23" s="20"/>
-      <c r="C23" s="45">
+      <c r="C23" s="44">
         <v>7</v>
       </c>
-      <c r="D23" s="57"/>
-      <c r="E23" s="53"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="53"/>
-      <c r="H23" s="54" t="str">
+      <c r="D23" s="56"/>
+      <c r="E23" s="52"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="52"/>
+      <c r="H23" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I23" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I23" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J23" s="6"/>
       <c r="L23" s="6"/>
-      <c r="M23" s="45">
+      <c r="M23" s="44">
         <v>7</v>
       </c>
-      <c r="N23" s="52">
+      <c r="N23" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O23" s="53">
+        <v/>
+      </c>
+      <c r="O23" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P23" s="52">
+        <v/>
+      </c>
+      <c r="P23" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q23" s="53">
+        <v/>
+      </c>
+      <c r="Q23" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R23" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R23" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S23" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S23" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T23" s="27"/>
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B24" s="20"/>
-      <c r="C24" s="45">
+      <c r="C24" s="44">
         <v>8</v>
       </c>
-      <c r="D24" s="52"/>
-      <c r="E24" s="53"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="53"/>
-      <c r="H24" s="54" t="str">
+      <c r="D24" s="51"/>
+      <c r="E24" s="52"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I24" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I24" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J24" s="6"/>
       <c r="L24" s="6"/>
-      <c r="M24" s="45">
+      <c r="M24" s="44">
         <v>8</v>
       </c>
-      <c r="N24" s="52">
+      <c r="N24" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O24" s="53">
+        <v/>
+      </c>
+      <c r="O24" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P24" s="52">
+        <v/>
+      </c>
+      <c r="P24" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q24" s="53">
+        <v/>
+      </c>
+      <c r="Q24" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R24" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R24" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S24" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S24" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T24" s="27"/>
     </row>
     <row r="25" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B25" s="20"/>
-      <c r="C25" s="45">
+      <c r="C25" s="44">
         <v>9</v>
       </c>
-      <c r="D25" s="52"/>
-      <c r="E25" s="53"/>
-      <c r="F25" s="52"/>
-      <c r="G25" s="53"/>
-      <c r="H25" s="54" t="str">
+      <c r="D25" s="51"/>
+      <c r="E25" s="52"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="52"/>
+      <c r="H25" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I25" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I25" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J25" s="6"/>
       <c r="L25" s="6"/>
-      <c r="M25" s="45">
+      <c r="M25" s="44">
         <v>9</v>
       </c>
-      <c r="N25" s="52">
+      <c r="N25" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O25" s="53">
+        <v/>
+      </c>
+      <c r="O25" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P25" s="52">
+        <v/>
+      </c>
+      <c r="P25" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q25" s="53">
+        <v/>
+      </c>
+      <c r="Q25" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R25" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R25" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S25" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S25" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T25" s="27"/>
     </row>
     <row r="26" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B26" s="20"/>
-      <c r="C26" s="45">
+      <c r="C26" s="44">
         <v>10</v>
       </c>
-      <c r="D26" s="52"/>
-      <c r="E26" s="53"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="53"/>
-      <c r="H26" s="54" t="str">
+      <c r="D26" s="51"/>
+      <c r="E26" s="52"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I26" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I26" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J26" s="6"/>
       <c r="L26" s="6"/>
-      <c r="M26" s="45">
+      <c r="M26" s="44">
         <v>10</v>
       </c>
-      <c r="N26" s="52">
+      <c r="N26" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O26" s="53">
+        <v/>
+      </c>
+      <c r="O26" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P26" s="52">
+        <v/>
+      </c>
+      <c r="P26" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q26" s="53">
+        <v/>
+      </c>
+      <c r="Q26" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R26" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R26" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S26" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S26" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T26" s="27"/>
     </row>
     <row r="27" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B27" s="20"/>
-      <c r="C27" s="45">
+      <c r="C27" s="44">
         <v>11</v>
       </c>
-      <c r="D27" s="52"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="52"/>
-      <c r="G27" s="53"/>
-      <c r="H27" s="54" t="str">
+      <c r="D27" s="51"/>
+      <c r="E27" s="52"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="52"/>
+      <c r="H27" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I27" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I27" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J27" s="6"/>
       <c r="L27" s="6"/>
-      <c r="M27" s="45">
+      <c r="M27" s="44">
         <v>11</v>
       </c>
-      <c r="N27" s="52">
+      <c r="N27" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O27" s="53">
+        <v/>
+      </c>
+      <c r="O27" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P27" s="52">
+        <v/>
+      </c>
+      <c r="P27" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q27" s="53">
+        <v/>
+      </c>
+      <c r="Q27" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R27" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R27" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S27" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S27" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T27" s="27"/>
     </row>
     <row r="28" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B28" s="20"/>
-      <c r="C28" s="45">
+      <c r="C28" s="44">
         <v>12</v>
       </c>
-      <c r="D28" s="58"/>
-      <c r="E28" s="59"/>
-      <c r="F28" s="58"/>
-      <c r="G28" s="59"/>
-      <c r="H28" s="54" t="str">
+      <c r="D28" s="57"/>
+      <c r="E28" s="58"/>
+      <c r="F28" s="57"/>
+      <c r="G28" s="58"/>
+      <c r="H28" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I28" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I28" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J28" s="13"/>
       <c r="K28" s="2"/>
       <c r="L28" s="6"/>
-      <c r="M28" s="45">
+      <c r="M28" s="44">
         <v>12</v>
       </c>
-      <c r="N28" s="52">
+      <c r="N28" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O28" s="53">
+        <v/>
+      </c>
+      <c r="O28" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P28" s="52">
+        <v/>
+      </c>
+      <c r="P28" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q28" s="53">
+        <v/>
+      </c>
+      <c r="Q28" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R28" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R28" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S28" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S28" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T28" s="27"/>
     </row>
     <row r="29" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B29" s="20"/>
-      <c r="C29" s="45">
+      <c r="C29" s="44">
         <v>13</v>
       </c>
-      <c r="D29" s="52"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="52"/>
-      <c r="G29" s="53"/>
-      <c r="H29" s="54" t="str">
+      <c r="D29" s="51"/>
+      <c r="E29" s="52"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="52"/>
+      <c r="H29" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I29" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I29" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J29" s="6"/>
       <c r="L29" s="6"/>
-      <c r="M29" s="45">
+      <c r="M29" s="44">
         <v>13</v>
       </c>
-      <c r="N29" s="52">
+      <c r="N29" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O29" s="53">
+        <v/>
+      </c>
+      <c r="O29" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P29" s="52">
+        <v/>
+      </c>
+      <c r="P29" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q29" s="53">
+        <v/>
+      </c>
+      <c r="Q29" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R29" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R29" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S29" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S29" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T29" s="27"/>
     </row>
     <row r="30" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B30" s="20"/>
-      <c r="C30" s="45">
+      <c r="C30" s="44">
         <v>14</v>
       </c>
-      <c r="D30" s="57"/>
-      <c r="E30" s="53"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="53"/>
-      <c r="H30" s="54" t="str">
+      <c r="D30" s="56"/>
+      <c r="E30" s="52"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="52"/>
+      <c r="H30" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I30" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I30" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J30" s="6"/>
       <c r="L30" s="6"/>
-      <c r="M30" s="45">
+      <c r="M30" s="44">
         <v>14</v>
       </c>
-      <c r="N30" s="52">
+      <c r="N30" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O30" s="53">
+        <v/>
+      </c>
+      <c r="O30" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P30" s="52">
+        <v/>
+      </c>
+      <c r="P30" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q30" s="53">
+        <v/>
+      </c>
+      <c r="Q30" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R30" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R30" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S30" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S30" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T30" s="27"/>
     </row>
     <row r="31" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B31" s="20"/>
-      <c r="C31" s="45">
+      <c r="C31" s="44">
         <v>15</v>
       </c>
-      <c r="D31" s="52"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="52"/>
-      <c r="G31" s="53"/>
-      <c r="H31" s="54" t="str">
+      <c r="D31" s="51"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="52"/>
+      <c r="H31" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I31" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I31" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J31" s="6"/>
       <c r="L31" s="6"/>
-      <c r="M31" s="45">
+      <c r="M31" s="44">
         <v>15</v>
       </c>
-      <c r="N31" s="52">
+      <c r="N31" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O31" s="53">
+        <v/>
+      </c>
+      <c r="O31" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P31" s="52">
+        <v/>
+      </c>
+      <c r="P31" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q31" s="53">
+        <v/>
+      </c>
+      <c r="Q31" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R31" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R31" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S31" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S31" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T31" s="27"/>
     </row>
     <row r="32" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B32" s="20"/>
-      <c r="C32" s="45">
+      <c r="C32" s="44">
         <v>16</v>
       </c>
-      <c r="D32" s="52"/>
-      <c r="E32" s="53"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="53"/>
-      <c r="H32" s="54" t="str">
+      <c r="D32" s="51"/>
+      <c r="E32" s="52"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="52"/>
+      <c r="H32" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I32" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I32" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J32" s="6"/>
       <c r="L32" s="6"/>
-      <c r="M32" s="45">
+      <c r="M32" s="44">
         <v>16</v>
       </c>
-      <c r="N32" s="52">
+      <c r="N32" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O32" s="53">
+        <v/>
+      </c>
+      <c r="O32" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P32" s="52">
+        <v/>
+      </c>
+      <c r="P32" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q32" s="53">
+        <v/>
+      </c>
+      <c r="Q32" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R32" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R32" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S32" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S32" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T32" s="27"/>
     </row>
     <row r="33" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B33" s="20"/>
-      <c r="C33" s="45">
+      <c r="C33" s="44">
         <v>17</v>
       </c>
-      <c r="D33" s="52"/>
-      <c r="E33" s="53"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="53"/>
-      <c r="H33" s="54" t="str">
+      <c r="D33" s="51"/>
+      <c r="E33" s="52"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="52"/>
+      <c r="H33" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I33" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I33" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J33" s="6"/>
       <c r="L33" s="6"/>
-      <c r="M33" s="45">
+      <c r="M33" s="44">
         <v>17</v>
       </c>
-      <c r="N33" s="52">
+      <c r="N33" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O33" s="53">
+        <v/>
+      </c>
+      <c r="O33" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P33" s="52">
+        <v/>
+      </c>
+      <c r="P33" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q33" s="53">
+        <v/>
+      </c>
+      <c r="Q33" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R33" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R33" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S33" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S33" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T33" s="27"/>
     </row>
     <row r="34" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B34" s="20"/>
-      <c r="C34" s="45">
+      <c r="C34" s="44">
         <v>18</v>
       </c>
-      <c r="D34" s="52"/>
-      <c r="E34" s="53"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="53"/>
-      <c r="H34" s="54" t="str">
+      <c r="D34" s="51"/>
+      <c r="E34" s="52"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="52"/>
+      <c r="H34" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I34" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I34" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J34" s="6"/>
       <c r="L34" s="6"/>
-      <c r="M34" s="45">
+      <c r="M34" s="44">
         <v>18</v>
       </c>
-      <c r="N34" s="52">
+      <c r="N34" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O34" s="53">
+        <v/>
+      </c>
+      <c r="O34" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P34" s="52">
+        <v/>
+      </c>
+      <c r="P34" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q34" s="53">
+        <v/>
+      </c>
+      <c r="Q34" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R34" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R34" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S34" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S34" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T34" s="27"/>
     </row>
     <row r="35" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B35" s="20"/>
-      <c r="C35" s="45">
+      <c r="C35" s="44">
         <v>19</v>
       </c>
-      <c r="D35" s="52"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="53"/>
-      <c r="H35" s="54" t="str">
+      <c r="D35" s="51"/>
+      <c r="E35" s="52"/>
+      <c r="F35" s="51"/>
+      <c r="G35" s="52"/>
+      <c r="H35" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I35" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I35" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J35" s="6"/>
       <c r="L35" s="6"/>
-      <c r="M35" s="45">
+      <c r="M35" s="44">
         <v>19</v>
       </c>
-      <c r="N35" s="52">
+      <c r="N35" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O35" s="53">
+        <v/>
+      </c>
+      <c r="O35" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P35" s="52">
+        <v/>
+      </c>
+      <c r="P35" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q35" s="53">
+        <v/>
+      </c>
+      <c r="Q35" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R35" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R35" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S35" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S35" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T35" s="27"/>
     </row>
     <row r="36" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B36" s="20"/>
-      <c r="C36" s="45">
+      <c r="C36" s="44">
         <v>20</v>
       </c>
-      <c r="D36" s="52"/>
-      <c r="E36" s="53"/>
-      <c r="F36" s="52"/>
-      <c r="G36" s="53"/>
-      <c r="H36" s="54" t="str">
+      <c r="D36" s="51"/>
+      <c r="E36" s="52"/>
+      <c r="F36" s="51"/>
+      <c r="G36" s="52"/>
+      <c r="H36" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I36" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I36" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J36" s="6"/>
       <c r="L36" s="6"/>
-      <c r="M36" s="45">
+      <c r="M36" s="44">
         <v>20</v>
       </c>
-      <c r="N36" s="52">
+      <c r="N36" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O36" s="53">
+        <v/>
+      </c>
+      <c r="O36" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P36" s="52">
+        <v/>
+      </c>
+      <c r="P36" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q36" s="53">
+        <v/>
+      </c>
+      <c r="Q36" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R36" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R36" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S36" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S36" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T36" s="27"/>
     </row>
     <row r="37" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B37" s="20"/>
-      <c r="C37" s="45">
+      <c r="C37" s="44">
         <v>21</v>
       </c>
-      <c r="D37" s="57"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="53"/>
-      <c r="H37" s="54" t="str">
+      <c r="D37" s="56"/>
+      <c r="E37" s="52"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="52"/>
+      <c r="H37" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I37" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I37" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J37" s="6"/>
       <c r="L37" s="6"/>
-      <c r="M37" s="45">
+      <c r="M37" s="44">
         <v>21</v>
       </c>
-      <c r="N37" s="52">
+      <c r="N37" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O37" s="53">
+        <v/>
+      </c>
+      <c r="O37" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P37" s="52">
+        <v/>
+      </c>
+      <c r="P37" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q37" s="53">
+        <v/>
+      </c>
+      <c r="Q37" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R37" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R37" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S37" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S37" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T37" s="27"/>
     </row>
     <row r="38" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B38" s="20"/>
-      <c r="C38" s="45">
+      <c r="C38" s="44">
         <v>22</v>
       </c>
-      <c r="D38" s="52"/>
-      <c r="E38" s="53"/>
-      <c r="F38" s="52"/>
-      <c r="G38" s="53"/>
-      <c r="H38" s="54" t="str">
+      <c r="D38" s="51"/>
+      <c r="E38" s="52"/>
+      <c r="F38" s="51"/>
+      <c r="G38" s="52"/>
+      <c r="H38" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I38" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I38" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J38" s="6"/>
       <c r="L38" s="6"/>
-      <c r="M38" s="45">
+      <c r="M38" s="44">
         <v>22</v>
       </c>
-      <c r="N38" s="52">
+      <c r="N38" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O38" s="53">
+        <v/>
+      </c>
+      <c r="O38" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P38" s="52">
+        <v/>
+      </c>
+      <c r="P38" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q38" s="53">
+        <v/>
+      </c>
+      <c r="Q38" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R38" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R38" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S38" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S38" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T38" s="27"/>
     </row>
     <row r="39" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B39" s="20"/>
-      <c r="C39" s="45">
+      <c r="C39" s="44">
         <v>23</v>
       </c>
-      <c r="D39" s="52"/>
-      <c r="E39" s="53"/>
-      <c r="F39" s="52"/>
-      <c r="G39" s="53"/>
-      <c r="H39" s="54" t="str">
+      <c r="D39" s="51"/>
+      <c r="E39" s="52"/>
+      <c r="F39" s="51"/>
+      <c r="G39" s="52"/>
+      <c r="H39" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I39" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I39" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J39" s="6"/>
       <c r="L39" s="6"/>
-      <c r="M39" s="45">
+      <c r="M39" s="44">
         <v>23</v>
       </c>
-      <c r="N39" s="52">
+      <c r="N39" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O39" s="53">
+        <v/>
+      </c>
+      <c r="O39" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P39" s="52">
+        <v/>
+      </c>
+      <c r="P39" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q39" s="53">
+        <v/>
+      </c>
+      <c r="Q39" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R39" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R39" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S39" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S39" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T39" s="27"/>
     </row>
     <row r="40" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B40" s="20"/>
-      <c r="C40" s="45">
+      <c r="C40" s="44">
         <v>24</v>
       </c>
-      <c r="D40" s="52"/>
-      <c r="E40" s="53"/>
-      <c r="F40" s="52"/>
-      <c r="G40" s="53"/>
-      <c r="H40" s="54" t="str">
+      <c r="D40" s="51"/>
+      <c r="E40" s="52"/>
+      <c r="F40" s="51"/>
+      <c r="G40" s="52"/>
+      <c r="H40" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I40" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I40" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J40" s="6"/>
       <c r="L40" s="6"/>
-      <c r="M40" s="45">
+      <c r="M40" s="44">
         <v>24</v>
       </c>
-      <c r="N40" s="52">
+      <c r="N40" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O40" s="53">
+        <v/>
+      </c>
+      <c r="O40" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P40" s="52">
+        <v/>
+      </c>
+      <c r="P40" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q40" s="53">
+        <v/>
+      </c>
+      <c r="Q40" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R40" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R40" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S40" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S40" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T40" s="27"/>
     </row>
     <row r="41" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B41" s="20"/>
-      <c r="C41" s="45">
+      <c r="C41" s="44">
         <v>25</v>
       </c>
-      <c r="D41" s="52"/>
-      <c r="E41" s="53"/>
-      <c r="F41" s="52"/>
-      <c r="G41" s="53"/>
-      <c r="H41" s="54" t="str">
+      <c r="D41" s="51"/>
+      <c r="E41" s="52"/>
+      <c r="F41" s="51"/>
+      <c r="G41" s="52"/>
+      <c r="H41" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I41" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I41" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J41" s="6"/>
       <c r="L41" s="6"/>
-      <c r="M41" s="45">
+      <c r="M41" s="44">
         <v>25</v>
       </c>
-      <c r="N41" s="52">
+      <c r="N41" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O41" s="53">
+        <v/>
+      </c>
+      <c r="O41" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P41" s="52">
+        <v/>
+      </c>
+      <c r="P41" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q41" s="53">
+        <v/>
+      </c>
+      <c r="Q41" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R41" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R41" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S41" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S41" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T41" s="27"/>
     </row>
     <row r="42" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B42" s="20"/>
-      <c r="C42" s="45">
+      <c r="C42" s="44">
         <v>26</v>
       </c>
-      <c r="D42" s="52"/>
-      <c r="E42" s="53"/>
-      <c r="F42" s="52"/>
-      <c r="G42" s="53"/>
-      <c r="H42" s="54" t="str">
+      <c r="D42" s="51"/>
+      <c r="E42" s="52"/>
+      <c r="F42" s="51"/>
+      <c r="G42" s="52"/>
+      <c r="H42" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I42" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I42" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J42" s="6"/>
       <c r="L42" s="6"/>
-      <c r="M42" s="45">
+      <c r="M42" s="44">
         <v>26</v>
       </c>
-      <c r="N42" s="52">
+      <c r="N42" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O42" s="53">
+        <v/>
+      </c>
+      <c r="O42" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P42" s="52">
+        <v/>
+      </c>
+      <c r="P42" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q42" s="53">
+        <v/>
+      </c>
+      <c r="Q42" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R42" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R42" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S42" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S42" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T42" s="27"/>
     </row>
     <row r="43" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B43" s="20"/>
-      <c r="C43" s="45">
+      <c r="C43" s="44">
         <v>27</v>
       </c>
-      <c r="D43" s="52"/>
-      <c r="E43" s="53"/>
-      <c r="F43" s="52"/>
-      <c r="G43" s="53"/>
-      <c r="H43" s="54" t="str">
+      <c r="D43" s="51"/>
+      <c r="E43" s="52"/>
+      <c r="F43" s="51"/>
+      <c r="G43" s="52"/>
+      <c r="H43" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I43" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I43" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J43" s="6"/>
       <c r="L43" s="6"/>
-      <c r="M43" s="45">
+      <c r="M43" s="44">
         <v>27</v>
       </c>
-      <c r="N43" s="52">
+      <c r="N43" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O43" s="53">
+        <v/>
+      </c>
+      <c r="O43" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P43" s="52">
+        <v/>
+      </c>
+      <c r="P43" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q43" s="53">
+        <v/>
+      </c>
+      <c r="Q43" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R43" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R43" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S43" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S43" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T43" s="27"/>
     </row>
     <row r="44" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B44" s="20"/>
-      <c r="C44" s="45">
+      <c r="C44" s="44">
         <v>28</v>
       </c>
-      <c r="D44" s="57"/>
-      <c r="E44" s="53"/>
-      <c r="F44" s="52"/>
-      <c r="G44" s="53"/>
-      <c r="H44" s="54" t="str">
+      <c r="D44" s="56"/>
+      <c r="E44" s="52"/>
+      <c r="F44" s="51"/>
+      <c r="G44" s="52"/>
+      <c r="H44" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I44" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I44" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J44" s="6"/>
       <c r="L44" s="6"/>
-      <c r="M44" s="45">
+      <c r="M44" s="44">
         <v>28</v>
       </c>
-      <c r="N44" s="52">
+      <c r="N44" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O44" s="53">
+        <v/>
+      </c>
+      <c r="O44" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P44" s="52">
+        <v/>
+      </c>
+      <c r="P44" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q44" s="53">
+        <v/>
+      </c>
+      <c r="Q44" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R44" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R44" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S44" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S44" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T44" s="27"/>
     </row>
     <row r="45" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B45" s="20"/>
-      <c r="C45" s="45">
+      <c r="C45" s="44">
         <v>29</v>
       </c>
-      <c r="D45" s="52"/>
-      <c r="E45" s="53"/>
-      <c r="F45" s="52"/>
-      <c r="G45" s="53"/>
-      <c r="H45" s="54" t="str">
+      <c r="D45" s="51"/>
+      <c r="E45" s="52"/>
+      <c r="F45" s="51"/>
+      <c r="G45" s="52"/>
+      <c r="H45" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I45" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I45" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J45" s="6"/>
       <c r="L45" s="6"/>
-      <c r="M45" s="45">
+      <c r="M45" s="44">
         <v>29</v>
       </c>
-      <c r="N45" s="52">
+      <c r="N45" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O45" s="53">
+        <v/>
+      </c>
+      <c r="O45" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P45" s="52">
+        <v/>
+      </c>
+      <c r="P45" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q45" s="53">
+        <v/>
+      </c>
+      <c r="Q45" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R45" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R45" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S45" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S45" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T45" s="27"/>
     </row>
     <row r="46" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B46" s="20"/>
-      <c r="C46" s="45">
+      <c r="C46" s="44">
         <v>30</v>
       </c>
-      <c r="D46" s="52"/>
-      <c r="E46" s="53"/>
-      <c r="F46" s="52"/>
-      <c r="G46" s="53"/>
-      <c r="H46" s="54" t="str">
+      <c r="D46" s="51"/>
+      <c r="E46" s="52"/>
+      <c r="F46" s="51"/>
+      <c r="G46" s="52"/>
+      <c r="H46" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I46" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I46" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J46" s="6"/>
       <c r="L46" s="6"/>
-      <c r="M46" s="45">
+      <c r="M46" s="44">
         <v>30</v>
       </c>
-      <c r="N46" s="52">
+      <c r="N46" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O46" s="53">
+        <v/>
+      </c>
+      <c r="O46" s="52" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P46" s="52">
+        <v/>
+      </c>
+      <c r="P46" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q46" s="53">
+        <v/>
+      </c>
+      <c r="Q46" s="52" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R46" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R46" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S46" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S46" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T46" s="27"/>
     </row>
     <row r="47" spans="2:20" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B47" s="20"/>
-      <c r="C47" s="51">
+      <c r="C47" s="50">
         <v>31</v>
       </c>
-      <c r="D47" s="52"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="52"/>
-      <c r="G47" s="60"/>
-      <c r="H47" s="54" t="str">
+      <c r="D47" s="51"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="51"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="I47" s="56" t="str">
+        <v/>
+      </c>
+      <c r="I47" s="55" t="str">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="J47" s="6"/>
       <c r="L47" s="6"/>
-      <c r="M47" s="51">
+      <c r="M47" s="50">
         <v>31</v>
       </c>
-      <c r="N47" s="52">
+      <c r="N47" s="51" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O47" s="53">
+        <v/>
+      </c>
+      <c r="O47" s="59" t="str">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P47" s="52">
+        <v/>
+      </c>
+      <c r="P47" s="51" t="str">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q47" s="53">
+        <v/>
+      </c>
+      <c r="Q47" s="59" t="str">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R47" s="54" t="str">
+        <v/>
+      </c>
+      <c r="R47" s="53" t="str">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-      <c r="S47" s="55" t="str">
+        <v/>
+      </c>
+      <c r="S47" s="54" t="str">
         <f t="shared" si="8"/>
-        <v>-</v>
+        <v/>
       </c>
       <c r="T47" s="27"/>
     </row>
@@ -2902,36 +2908,36 @@
       <c r="B48" s="20"/>
       <c r="C48" s="4"/>
       <c r="D48" s="5"/>
-      <c r="E48" s="42"/>
-      <c r="F48" s="42"/>
-      <c r="G48" s="43" t="s">
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="H48" s="61">
-        <f>SUM(H17:H47)</f>
-        <v>0</v>
-      </c>
-      <c r="I48" s="62">
-        <f>SUM(I17:I47)</f>
-        <v>0</v>
+      <c r="H48" s="60" t="str">
+        <f>IF(SUM(H17:H47)&gt;0,SUM(H17:H47),"")</f>
+        <v/>
+      </c>
+      <c r="I48" s="61" t="str">
+        <f>IF(SUM(I17:I47)&gt;0,SUM(I17:I47),"")</f>
+        <v/>
       </c>
       <c r="J48" s="16"/>
       <c r="K48" s="14"/>
       <c r="L48" s="7"/>
       <c r="M48" s="4"/>
       <c r="N48" s="5"/>
-      <c r="O48" s="42"/>
-      <c r="P48" s="42"/>
-      <c r="Q48" s="43" t="s">
+      <c r="O48" s="41"/>
+      <c r="P48" s="41"/>
+      <c r="Q48" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="R48" s="61">
-        <f>H48</f>
-        <v>0</v>
-      </c>
-      <c r="S48" s="62">
-        <f>I48</f>
-        <v>0</v>
+      <c r="R48" s="60" t="str">
+        <f>IF(H48="","",H48)</f>
+        <v/>
+      </c>
+      <c r="S48" s="61" t="str">
+        <f>IF(I48="","",I48)</f>
+        <v/>
       </c>
       <c r="T48" s="27"/>
     </row>
@@ -2943,86 +2949,86 @@
     </row>
     <row r="50" spans="2:20" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="20"/>
-      <c r="C50" s="83" t="s">
+      <c r="C50" s="82" t="s">
         <v>19</v>
       </c>
-      <c r="D50" s="83"/>
-      <c r="E50" s="83"/>
-      <c r="F50" s="83"/>
-      <c r="G50" s="83"/>
-      <c r="H50" s="83"/>
-      <c r="I50" s="83"/>
+      <c r="D50" s="82"/>
+      <c r="E50" s="82"/>
+      <c r="F50" s="82"/>
+      <c r="G50" s="82"/>
+      <c r="H50" s="82"/>
+      <c r="I50" s="82"/>
       <c r="J50" s="15"/>
       <c r="L50" s="12"/>
-      <c r="M50" s="83" t="s">
+      <c r="M50" s="82" t="s">
         <v>19</v>
       </c>
-      <c r="N50" s="83"/>
-      <c r="O50" s="83"/>
-      <c r="P50" s="83"/>
-      <c r="Q50" s="83"/>
-      <c r="R50" s="83"/>
-      <c r="S50" s="83"/>
+      <c r="N50" s="82"/>
+      <c r="O50" s="82"/>
+      <c r="P50" s="82"/>
+      <c r="Q50" s="82"/>
+      <c r="R50" s="82"/>
+      <c r="S50" s="82"/>
       <c r="T50" s="27"/>
     </row>
     <row r="51" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B51" s="20"/>
-      <c r="C51" s="83"/>
-      <c r="D51" s="83"/>
-      <c r="E51" s="83"/>
-      <c r="F51" s="83"/>
-      <c r="G51" s="83"/>
-      <c r="H51" s="83"/>
-      <c r="I51" s="83"/>
+      <c r="C51" s="82"/>
+      <c r="D51" s="82"/>
+      <c r="E51" s="82"/>
+      <c r="F51" s="82"/>
+      <c r="G51" s="82"/>
+      <c r="H51" s="82"/>
+      <c r="I51" s="82"/>
       <c r="J51" s="15"/>
       <c r="L51" s="12"/>
-      <c r="M51" s="83"/>
-      <c r="N51" s="83"/>
-      <c r="O51" s="83"/>
-      <c r="P51" s="83"/>
-      <c r="Q51" s="83"/>
-      <c r="R51" s="83"/>
-      <c r="S51" s="83"/>
+      <c r="M51" s="82"/>
+      <c r="N51" s="82"/>
+      <c r="O51" s="82"/>
+      <c r="P51" s="82"/>
+      <c r="Q51" s="82"/>
+      <c r="R51" s="82"/>
+      <c r="S51" s="82"/>
       <c r="T51" s="27"/>
     </row>
     <row r="52" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B52" s="20"/>
-      <c r="C52" s="83"/>
-      <c r="D52" s="83"/>
-      <c r="E52" s="83"/>
-      <c r="F52" s="83"/>
-      <c r="G52" s="83"/>
-      <c r="H52" s="83"/>
-      <c r="I52" s="83"/>
+      <c r="C52" s="82"/>
+      <c r="D52" s="82"/>
+      <c r="E52" s="82"/>
+      <c r="F52" s="82"/>
+      <c r="G52" s="82"/>
+      <c r="H52" s="82"/>
+      <c r="I52" s="82"/>
       <c r="J52" s="15"/>
       <c r="L52" s="12"/>
-      <c r="M52" s="83"/>
-      <c r="N52" s="83"/>
-      <c r="O52" s="83"/>
-      <c r="P52" s="83"/>
-      <c r="Q52" s="83"/>
-      <c r="R52" s="83"/>
-      <c r="S52" s="83"/>
+      <c r="M52" s="82"/>
+      <c r="N52" s="82"/>
+      <c r="O52" s="82"/>
+      <c r="P52" s="82"/>
+      <c r="Q52" s="82"/>
+      <c r="R52" s="82"/>
+      <c r="S52" s="82"/>
       <c r="T52" s="27"/>
     </row>
     <row r="53" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B53" s="20"/>
-      <c r="C53" s="83"/>
-      <c r="D53" s="83"/>
-      <c r="E53" s="83"/>
-      <c r="F53" s="83"/>
-      <c r="G53" s="83"/>
-      <c r="H53" s="83"/>
-      <c r="I53" s="83"/>
+      <c r="C53" s="82"/>
+      <c r="D53" s="82"/>
+      <c r="E53" s="82"/>
+      <c r="F53" s="82"/>
+      <c r="G53" s="82"/>
+      <c r="H53" s="82"/>
+      <c r="I53" s="82"/>
       <c r="J53" s="15"/>
       <c r="L53" s="12"/>
-      <c r="M53" s="83"/>
-      <c r="N53" s="83"/>
-      <c r="O53" s="83"/>
-      <c r="P53" s="83"/>
-      <c r="Q53" s="83"/>
-      <c r="R53" s="83"/>
-      <c r="S53" s="83"/>
+      <c r="M53" s="82"/>
+      <c r="N53" s="82"/>
+      <c r="O53" s="82"/>
+      <c r="P53" s="82"/>
+      <c r="Q53" s="82"/>
+      <c r="R53" s="82"/>
+      <c r="S53" s="82"/>
       <c r="T53" s="27"/>
     </row>
     <row r="54" spans="2:20" x14ac:dyDescent="0.2">
@@ -3033,77 +3039,77 @@
     </row>
     <row r="55" spans="2:20" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B55" s="20"/>
-      <c r="D55" s="80"/>
-      <c r="E55" s="80"/>
-      <c r="F55" s="80"/>
-      <c r="G55" s="80"/>
-      <c r="H55" s="80"/>
+      <c r="D55" s="79"/>
+      <c r="E55" s="79"/>
+      <c r="F55" s="79"/>
+      <c r="G55" s="79"/>
+      <c r="H55" s="79"/>
       <c r="J55" s="15"/>
       <c r="L55" s="12"/>
-      <c r="N55" s="80">
-        <f>D55</f>
-        <v>0</v>
-      </c>
-      <c r="O55" s="80"/>
-      <c r="P55" s="80"/>
-      <c r="Q55" s="80"/>
-      <c r="R55" s="80"/>
+      <c r="N55" s="79" t="str">
+        <f>IF(D55="","",D55)</f>
+        <v/>
+      </c>
+      <c r="O55" s="79"/>
+      <c r="P55" s="79"/>
+      <c r="Q55" s="79"/>
+      <c r="R55" s="79"/>
       <c r="T55" s="27"/>
     </row>
     <row r="56" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B56" s="20"/>
-      <c r="D56" s="39"/>
-      <c r="E56" s="39"/>
-      <c r="F56" s="39"/>
-      <c r="G56" s="39"/>
-      <c r="H56" s="39"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="38"/>
+      <c r="F56" s="38"/>
+      <c r="G56" s="38"/>
+      <c r="H56" s="38"/>
       <c r="J56" s="15"/>
       <c r="L56" s="20"/>
-      <c r="N56" s="39"/>
-      <c r="O56" s="39"/>
-      <c r="P56" s="39"/>
-      <c r="Q56" s="39"/>
-      <c r="R56" s="39"/>
+      <c r="N56" s="38"/>
+      <c r="O56" s="38"/>
+      <c r="P56" s="38"/>
+      <c r="Q56" s="38"/>
+      <c r="R56" s="38"/>
       <c r="T56" s="15"/>
     </row>
     <row r="57" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B57" s="20"/>
-      <c r="D57" s="39"/>
-      <c r="E57" s="39"/>
-      <c r="F57" s="39"/>
-      <c r="G57" s="39"/>
-      <c r="H57" s="39"/>
+      <c r="D57" s="38"/>
+      <c r="E57" s="38"/>
+      <c r="F57" s="38"/>
+      <c r="G57" s="38"/>
+      <c r="H57" s="38"/>
       <c r="J57" s="15"/>
       <c r="L57" s="20"/>
-      <c r="N57" s="39"/>
-      <c r="O57" s="39"/>
-      <c r="P57" s="39"/>
-      <c r="Q57" s="39"/>
-      <c r="R57" s="39"/>
+      <c r="N57" s="38"/>
+      <c r="O57" s="38"/>
+      <c r="P57" s="38"/>
+      <c r="Q57" s="38"/>
+      <c r="R57" s="38"/>
       <c r="T57" s="15"/>
     </row>
     <row r="58" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B58" s="20"/>
-      <c r="C58" s="69" t="s">
+      <c r="C58" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="D58" s="69"/>
-      <c r="E58" s="69"/>
-      <c r="F58" s="69"/>
-      <c r="G58" s="69"/>
-      <c r="H58" s="69"/>
-      <c r="I58" s="69"/>
+      <c r="D58" s="68"/>
+      <c r="E58" s="68"/>
+      <c r="F58" s="68"/>
+      <c r="G58" s="68"/>
+      <c r="H58" s="68"/>
+      <c r="I58" s="68"/>
       <c r="J58" s="15"/>
       <c r="L58" s="20"/>
-      <c r="M58" s="69" t="s">
+      <c r="M58" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="N58" s="69"/>
-      <c r="O58" s="69"/>
-      <c r="P58" s="69"/>
-      <c r="Q58" s="69"/>
-      <c r="R58" s="69"/>
-      <c r="S58" s="69"/>
+      <c r="N58" s="68"/>
+      <c r="O58" s="68"/>
+      <c r="P58" s="68"/>
+      <c r="Q58" s="68"/>
+      <c r="R58" s="68"/>
+      <c r="S58" s="68"/>
       <c r="T58" s="15"/>
     </row>
     <row r="59" spans="2:20" x14ac:dyDescent="0.2">
@@ -3120,79 +3126,79 @@
     </row>
     <row r="61" spans="2:20" ht="10.8" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B61" s="20"/>
-      <c r="D61" s="72"/>
-      <c r="E61" s="72"/>
-      <c r="F61" s="72"/>
-      <c r="G61" s="72"/>
-      <c r="H61" s="72"/>
+      <c r="D61" s="71"/>
+      <c r="E61" s="71"/>
+      <c r="F61" s="71"/>
+      <c r="G61" s="71"/>
+      <c r="H61" s="71"/>
       <c r="J61" s="15"/>
       <c r="L61" s="20"/>
-      <c r="N61" s="72">
-        <f>D61</f>
-        <v>0</v>
-      </c>
-      <c r="O61" s="72"/>
-      <c r="P61" s="72"/>
-      <c r="Q61" s="72"/>
-      <c r="R61" s="72"/>
+      <c r="N61" s="71" t="str">
+        <f>IF(D61="","",D61)</f>
+        <v/>
+      </c>
+      <c r="O61" s="71"/>
+      <c r="P61" s="71"/>
+      <c r="Q61" s="71"/>
+      <c r="R61" s="71"/>
       <c r="T61" s="15"/>
     </row>
     <row r="62" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B62" s="20"/>
-      <c r="D62" s="63" t="s">
+      <c r="D62" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="E62" s="64"/>
-      <c r="F62" s="64"/>
-      <c r="G62" s="64"/>
-      <c r="H62" s="64"/>
+      <c r="E62" s="63"/>
+      <c r="F62" s="63"/>
+      <c r="G62" s="63"/>
+      <c r="H62" s="63"/>
       <c r="I62" s="8"/>
       <c r="J62" s="22"/>
       <c r="K62" s="8"/>
       <c r="L62" s="20"/>
-      <c r="N62" s="63" t="s">
+      <c r="N62" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="O62" s="64"/>
-      <c r="P62" s="64"/>
-      <c r="Q62" s="64"/>
-      <c r="R62" s="64"/>
+      <c r="O62" s="63"/>
+      <c r="P62" s="63"/>
+      <c r="Q62" s="63"/>
+      <c r="R62" s="63"/>
       <c r="S62" s="8"/>
       <c r="T62" s="22"/>
     </row>
     <row r="63" spans="2:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B63" s="23"/>
       <c r="C63" s="10"/>
-      <c r="D63" s="46"/>
-      <c r="E63" s="47"/>
-      <c r="F63" s="47"/>
-      <c r="G63" s="47"/>
-      <c r="H63" s="47"/>
-      <c r="I63" s="48"/>
-      <c r="J63" s="49"/>
+      <c r="D63" s="45"/>
+      <c r="E63" s="46"/>
+      <c r="F63" s="46"/>
+      <c r="G63" s="46"/>
+      <c r="H63" s="46"/>
+      <c r="I63" s="47"/>
+      <c r="J63" s="48"/>
       <c r="K63" s="8"/>
       <c r="L63" s="23"/>
       <c r="M63" s="10"/>
-      <c r="N63" s="46"/>
-      <c r="O63" s="47"/>
-      <c r="P63" s="47"/>
-      <c r="Q63" s="47"/>
-      <c r="R63" s="47"/>
-      <c r="S63" s="48"/>
-      <c r="T63" s="49"/>
+      <c r="N63" s="45"/>
+      <c r="O63" s="46"/>
+      <c r="P63" s="46"/>
+      <c r="Q63" s="46"/>
+      <c r="R63" s="46"/>
+      <c r="S63" s="47"/>
+      <c r="T63" s="48"/>
     </row>
     <row r="64" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="H64" s="65"/>
-      <c r="I64" s="65"/>
+      <c r="H64" s="64"/>
+      <c r="I64" s="64"/>
       <c r="J64" s="24"/>
       <c r="K64" s="24"/>
       <c r="L64" s="2"/>
-      <c r="R64" s="65"/>
-      <c r="S64" s="65"/>
+      <c r="R64" s="64"/>
+      <c r="S64" s="64"/>
       <c r="T64" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="42">
     <mergeCell ref="M13:O13"/>
     <mergeCell ref="D55:H55"/>
     <mergeCell ref="N55:R55"/>
@@ -3205,6 +3211,10 @@
     <mergeCell ref="M12:O12"/>
     <mergeCell ref="M50:S53"/>
     <mergeCell ref="C50:I53"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="R12:S12"/>
+    <mergeCell ref="R13:S13"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="M2:O2"/>
     <mergeCell ref="D5:H5"/>

</xml_diff>